<commit_message>
Show specific exams and SOL tests on the pacing calendar
Adds an editable exam/test date table to the Assessments tab and prints
each entry on its day in Year at a Glance (midyear and final exam
subjects, SOL test dates). Benchmark labels now read 'Benchmark'.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y9R7PeCARjWUDy39JuMJzQ
</commit_message>
<xml_diff>
--- a/english9-pacing/English9_PurpleGold_Pacing_2026-27.xlsx
+++ b/english9-pacing/English9_PurpleGold_Pacing_2026-27.xlsx
@@ -213,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -299,11 +299,16 @@
     <xf numFmtId="165" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -742,7 +747,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Assessments: where each midquarter, benchmark and LPA landed for each track, inside its testing window.</t>
+          <t>Assessments: where each midquarter, benchmark and LPA landed for each track, inside its testing window. Its yellow Exam table (columns H and I) lists midyear exams, final exams and SOL test dates; each one is printed on its day in Year at a Glance.</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1035,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="40" customHeight="1">
       <c r="A7" s="13" t="n"/>
       <c r="B7" s="13" t="n"/>
       <c r="C7" s="13" t="n"/>
@@ -1045,15 +1050,15 @@
       <c r="I7" s="13" t="n"/>
       <c r="J7" s="13" t="n"/>
       <c r="K7" s="15">
-        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,1),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,1),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,1),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="L7" s="16">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,2),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,2),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,2),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="M7" s="15">
-        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,3),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,3),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,3),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="N7" s="14" t="inlineStr">
@@ -1071,11 +1076,11 @@
       <c r="S7" s="13" t="n"/>
       <c r="T7" s="13" t="n"/>
       <c r="U7" s="15">
-        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,1),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,1),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,1),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="V7" s="16">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,2),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,2),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,2),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="W7" s="14" t="inlineStr">
@@ -1084,7 +1089,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="40" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
           <t>2</t>
@@ -1131,19 +1136,19 @@
         </is>
       </c>
       <c r="K8" s="16">
-        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,8),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,8),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,8),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="L8" s="15">
-        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,9),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,9),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,9),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="M8" s="16">
-        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,10),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,10),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,10),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="N8" s="15">
-        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,11),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,11),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,11),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="O8" s="14" t="inlineStr">
@@ -1157,23 +1162,23 @@
         </is>
       </c>
       <c r="R8" s="15">
-        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,5),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,5),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,5),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="S8" s="16">
-        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,6),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,6),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,6),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="T8" s="15">
-        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,7),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,7),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,7),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="U8" s="16">
-        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,8),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,8),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,8),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="V8" s="15">
-        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,9),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,9),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,9),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="W8" s="14" t="inlineStr">
@@ -1182,7 +1187,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="40" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
           <t>9</t>
@@ -1224,23 +1229,23 @@
         </is>
       </c>
       <c r="J9" s="16">
-        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,14),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,14),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,14),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="K9" s="15">
-        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,15),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,15),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,15),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="L9" s="16">
-        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,16),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,16),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,16),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="M9" s="15">
-        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,17),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,17),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,17),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="N9" s="16">
-        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,18),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,18),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,18),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="O9" s="14" t="inlineStr">
@@ -1254,19 +1259,19 @@
         </is>
       </c>
       <c r="R9" s="16">
-        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,12),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,12),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,12),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="S9" s="15">
-        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,13),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,13),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,13),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="T9" s="16">
-        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,14),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,14),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,14),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="U9" s="15">
-        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,15),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,15),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,15),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="V9" s="14" t="inlineStr">
@@ -1280,7 +1285,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="40" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
           <t>16</t>
@@ -1322,23 +1327,23 @@
         </is>
       </c>
       <c r="J10" s="15">
-        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,21),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,21),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,21),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="K10" s="16">
-        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,22),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,22),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,22),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="L10" s="15">
-        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,23),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,23),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,23),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="M10" s="16">
-        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,24),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,24),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,24),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="N10" s="15">
-        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,25),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,25),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,25),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="O10" s="14" t="inlineStr">
@@ -1352,23 +1357,23 @@
         </is>
       </c>
       <c r="R10" s="16">
-        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,19),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,19),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,19),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="S10" s="15">
-        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,20),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,20),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,20),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="T10" s="16">
-        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,21),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,21),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,21),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="U10" s="15">
-        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,22),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,22),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,22),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="V10" s="16">
-        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,23),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,23),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,23),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="W10" s="14" t="inlineStr">
@@ -1377,30 +1382,30 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="40" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
       <c r="B11" s="15">
-        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,24),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,24),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,8,24),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C11" s="16">
-        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,25),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,25),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,8,25),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="D11" s="15">
-        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,26),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,26),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,8,26),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="E11" s="16">
-        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,27),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,27),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,8,27),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="F11" s="15">
-        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,28),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,28),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,8,28),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="G11" s="14" t="inlineStr">
@@ -1414,15 +1419,15 @@
         </is>
       </c>
       <c r="J11" s="16">
-        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,28),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,28),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,28),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="K11" s="15">
-        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,29),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,29),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,29),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="L11" s="16">
-        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,30),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,30),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,30),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="M11" s="13" t="n"/>
@@ -1434,23 +1439,23 @@
         </is>
       </c>
       <c r="R11" s="15">
-        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,26),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,26),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,26),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="S11" s="16">
-        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,27),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,27),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,27),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="T11" s="15">
-        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,28),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,28),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,28),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="U11" s="16">
-        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,29),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,29),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,29),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="V11" s="15">
-        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,30),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,30),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,30),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="W11" s="14" t="inlineStr">
@@ -1459,14 +1464,14 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="40" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
       <c r="B12" s="16">
-        <f>"31"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,31),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"31"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,31),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,8,31),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C12" s="13" t="n"/>
@@ -1613,14 +1618,14 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="40" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="B16" s="16">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,2),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,2),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,2),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C16" s="14" t="inlineStr">
@@ -1629,15 +1634,15 @@
         </is>
       </c>
       <c r="D16" s="15">
-        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,4),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,4),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,4),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="E16" s="16">
-        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,5),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,5),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,5),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,6),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,6),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,6),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="G16" s="14" t="inlineStr">
@@ -1648,19 +1653,19 @@
       <c r="I16" s="13" t="n"/>
       <c r="J16" s="13" t="n"/>
       <c r="K16" s="15">
-        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,1),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,1),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,1),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="L16" s="16">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,2),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,2),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,2),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="M16" s="15">
-        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,3),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,3),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,3),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="N16" s="16">
-        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,4),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,4),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,4),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="O16" s="14" t="inlineStr">
@@ -1684,30 +1689,30 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="40" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
       <c r="B17" s="16">
-        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,9),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,9),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,9),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C17" s="15">
-        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,10),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,10),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,10),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="D17" s="16">
-        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,11),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,11),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,11),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="E17" s="15">
-        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,12),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,12),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,12),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="F17" s="16">
-        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,13),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,13),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,13),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="G17" s="14" t="inlineStr">
@@ -1721,23 +1726,23 @@
         </is>
       </c>
       <c r="J17" s="15">
-        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,7),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,7),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,7),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="K17" s="16">
-        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,8),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,8),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,8),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="L17" s="15">
-        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,9),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,9),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,9),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="M17" s="16">
-        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,10),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,10),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,10),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="N17" s="15">
-        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,11),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,11),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,11),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="O17" s="14" t="inlineStr">
@@ -1756,19 +1761,19 @@
         </is>
       </c>
       <c r="S17" s="15">
-        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,5),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,5),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,5),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="T17" s="16">
-        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,6),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,6),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,6),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="U17" s="15">
-        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,7),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,7),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,7),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="V17" s="16">
-        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,8),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,8),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,8),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="W17" s="14" t="inlineStr">
@@ -1777,30 +1782,30 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="28" customHeight="1">
+    <row r="18" ht="40" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
       <c r="B18" s="15">
-        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,16),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,16),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,16),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C18" s="16">
-        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,17),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,17),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,17),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="D18" s="15">
-        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,18),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,18),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,18),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="E18" s="16">
-        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,19),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,19),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,19),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="F18" s="15">
-        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,20),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,20),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,20),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="G18" s="14" t="inlineStr">
@@ -1814,23 +1819,23 @@
         </is>
       </c>
       <c r="J18" s="16">
-        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,14),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,14),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,14),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="K18" s="15">
-        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,15),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,15),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,15),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="L18" s="16">
-        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,16),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,16),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,16),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="M18" s="15">
-        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,17),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,17),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,17),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="N18" s="16">
-        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,18),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,18),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,18),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="O18" s="14" t="inlineStr">
@@ -1844,23 +1849,23 @@
         </is>
       </c>
       <c r="R18" s="15">
-        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,11),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,11),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,11),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="S18" s="16">
-        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,12),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,12),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,12),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="T18" s="15">
-        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,13),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,13),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,13),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="U18" s="16">
-        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,14),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,14),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,14),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="V18" s="15">
-        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,15),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,15),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,15),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="W18" s="14" t="inlineStr">
@@ -1869,18 +1874,18 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="40" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
       <c r="B19" s="16">
-        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,23),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,23),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,23),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C19" s="15">
-        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,24),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,24),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,24),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="D19" s="14" t="inlineStr">
@@ -1949,19 +1954,19 @@
         </is>
       </c>
       <c r="S19" s="16">
-        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,19),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,19),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,19),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="T19" s="17">
-        <f>"20"&amp;CHAR(10)&amp;IFERROR("P: "&amp;VLOOKUP(DATE(2027,1,20),Purple!$A:$J,10,FALSE),IFERROR("G: "&amp;VLOOKUP(DATE(2027,1,20),Gold!$A:$J,10,FALSE),"Exam"))</f>
+        <f>"20"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,1,20),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,1,20),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,20),Assessments!$H:$I,2,FALSE),CHAR(10)&amp;"Exam day")</f>
         <v/>
       </c>
       <c r="U19" s="17">
-        <f>"21"&amp;CHAR(10)&amp;IFERROR("P: "&amp;VLOOKUP(DATE(2027,1,21),Purple!$A:$J,10,FALSE),IFERROR("G: "&amp;VLOOKUP(DATE(2027,1,21),Gold!$A:$J,10,FALSE),"Exam"))</f>
+        <f>"21"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,1,21),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,1,21),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,21),Assessments!$H:$I,2,FALSE),CHAR(10)&amp;"Exam day")</f>
         <v/>
       </c>
       <c r="V19" s="17">
-        <f>"22"&amp;CHAR(10)&amp;IFERROR("P: "&amp;VLOOKUP(DATE(2027,1,22),Purple!$A:$J,10,FALSE),IFERROR("G: "&amp;VLOOKUP(DATE(2027,1,22),Gold!$A:$J,10,FALSE),"Exam"))</f>
+        <f>"22"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,1,22),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,1,22),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,22),Assessments!$H:$I,2,FALSE),CHAR(10)&amp;"Exam day")</f>
         <v/>
       </c>
       <c r="W19" s="14" t="inlineStr">
@@ -1970,14 +1975,14 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="40" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
       <c r="B20" s="16">
-        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,30),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,30),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,30),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C20" s="13" t="n"/>
@@ -2028,15 +2033,15 @@
         </is>
       </c>
       <c r="T20" s="15">
-        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,27),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,27),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,27),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="U20" s="16">
-        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,28),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,28),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,28),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="V20" s="15">
-        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,29),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,29),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,29),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="W20" s="14" t="inlineStr">
@@ -2045,7 +2050,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="28" customHeight="1">
+    <row r="21" ht="40" customHeight="1">
       <c r="A21" s="13" t="n"/>
       <c r="B21" s="13" t="n"/>
       <c r="C21" s="13" t="n"/>
@@ -2196,26 +2201,26 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="40" customHeight="1">
       <c r="A25" s="13" t="n"/>
       <c r="B25" s="16">
-        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,1),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,1),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,1),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C25" s="15">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,2),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,2),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,2),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="D25" s="16">
-        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,3),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,3),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,3),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="E25" s="15">
-        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,4),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,4),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,4),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="F25" s="16">
-        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,5),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,5),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,5),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="G25" s="14" t="inlineStr">
@@ -2225,23 +2230,23 @@
       </c>
       <c r="I25" s="13" t="n"/>
       <c r="J25" s="15">
-        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,1),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,1),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,1),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="K25" s="16">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,2),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,2),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,2),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="L25" s="15">
-        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,3),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,3),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,3),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="M25" s="16">
-        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,4),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,4),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,4),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="N25" s="18">
-        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,5),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,5),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,5),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="O25" s="14" t="inlineStr">
@@ -2254,11 +2259,11 @@
       <c r="S25" s="13" t="n"/>
       <c r="T25" s="13" t="n"/>
       <c r="U25" s="16">
-        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,1),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,1),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,1),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="V25" s="18">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,2),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,2),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,2),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="W25" s="14" t="inlineStr">
@@ -2267,30 +2272,30 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="28" customHeight="1">
+    <row r="26" ht="40" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
       <c r="B26" s="15">
-        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,8),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,8),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,8),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C26" s="16">
-        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,9),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,9),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,9),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="D26" s="15">
-        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,10),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,10),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,10),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="E26" s="16">
-        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,11),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,11),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,11),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="F26" s="15">
-        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,12),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,12),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,12),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="G26" s="14" t="inlineStr">
@@ -2304,23 +2309,23 @@
         </is>
       </c>
       <c r="J26" s="16">
-        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,8),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,8),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,8),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="K26" s="15">
-        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,9),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,9),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,9),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="L26" s="16">
-        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,10),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,10),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,10),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="M26" s="15">
-        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,11),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,11),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,11),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="N26" s="16">
-        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,12),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,12),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,12),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="O26" s="14" t="inlineStr">
@@ -2364,7 +2369,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="28" customHeight="1">
+    <row r="27" ht="40" customHeight="1">
       <c r="A27" s="14" t="inlineStr">
         <is>
           <t>14</t>
@@ -2376,19 +2381,19 @@
         </is>
       </c>
       <c r="C27" s="16">
-        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,16),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,16),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,16),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="D27" s="15">
-        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,17),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,17),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,17),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="E27" s="16">
-        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,18),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,18),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,18),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="F27" s="15">
-        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,19),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,19),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,19),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="G27" s="14" t="inlineStr">
@@ -2402,23 +2407,23 @@
         </is>
       </c>
       <c r="J27" s="15">
-        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,15),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,15),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,15),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="K27" s="16">
-        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,16),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,16),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,16),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="L27" s="15">
-        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,17),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,17),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,17),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="M27" s="16">
-        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,18),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,18),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,18),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="N27" s="15">
-        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,19),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,19),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,19),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="O27" s="14" t="inlineStr">
@@ -2437,19 +2442,19 @@
         </is>
       </c>
       <c r="S27" s="16">
-        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,13),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,13),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,13),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="T27" s="15">
-        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,14),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,14),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,14),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="U27" s="16">
-        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,15),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,15),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,15),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="V27" s="15">
-        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,16),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,16),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,16),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="W27" s="14" t="inlineStr">
@@ -2458,30 +2463,30 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="28" customHeight="1">
+    <row r="28" ht="40" customHeight="1">
       <c r="A28" s="14" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
       <c r="B28" s="16">
-        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,22),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,22),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,22),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C28" s="15">
-        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,23),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,23),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,23),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="D28" s="16">
-        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,24),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,24),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,24),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="E28" s="15">
-        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,25),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,25),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,25),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="F28" s="16">
-        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,26),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,26),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,26),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="G28" s="14" t="inlineStr">
@@ -2495,23 +2500,23 @@
         </is>
       </c>
       <c r="J28" s="16">
-        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,22),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,22),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,22),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="K28" s="15">
-        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,23),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,23),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,23),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="L28" s="16">
-        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,24),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,24),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,24),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="M28" s="15">
-        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,25),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,25),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,25),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="N28" s="16">
-        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,26),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,26),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,26),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="O28" s="14" t="inlineStr">
@@ -2525,23 +2530,23 @@
         </is>
       </c>
       <c r="R28" s="16">
-        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,19),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,19),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,19),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="S28" s="15">
-        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,20),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,20),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,20),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="T28" s="16">
-        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,21),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,21),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,21),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="U28" s="15">
-        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,22),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,22),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,22),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="V28" s="16">
-        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,23),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,23),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,23),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="W28" s="14" t="inlineStr">
@@ -2550,7 +2555,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="40" customHeight="1">
       <c r="A29" s="14" t="inlineStr">
         <is>
           <t>28</t>
@@ -2568,15 +2573,15 @@
         </is>
       </c>
       <c r="J29" s="15">
-        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,29),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,29),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,29),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="K29" s="16">
-        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,30),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,30),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,30),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="L29" s="15">
-        <f>"31"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,31),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"31"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,31),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,31),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="M29" s="13" t="n"/>
@@ -2588,28 +2593,28 @@
         </is>
       </c>
       <c r="R29" s="15">
-        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,26),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,26),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,26),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="S29" s="16">
-        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,27),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,27),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,27),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="T29" s="15">
-        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,28),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,28),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,28),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="U29" s="16">
-        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,29),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,29),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,29),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="V29" s="15">
-        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,30),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,30),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,30),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="W29" s="13" t="n"/>
     </row>
-    <row r="30" ht="28" customHeight="1">
+    <row r="30" ht="40" customHeight="1">
       <c r="A30" s="13" t="n"/>
       <c r="B30" s="13" t="n"/>
       <c r="C30" s="13" t="n"/>
@@ -2716,7 +2721,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="28" customHeight="1">
+    <row r="34" ht="40" customHeight="1">
       <c r="A34" s="13" t="n"/>
       <c r="B34" s="13" t="n"/>
       <c r="C34" s="13" t="n"/>
@@ -2731,19 +2736,19 @@
       <c r="I34" s="13" t="n"/>
       <c r="J34" s="13" t="n"/>
       <c r="K34" s="16">
-        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,6,1),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,6,1),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,6,1),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="L34" s="15">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,6,2),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,6,2),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,6,2),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="M34" s="16">
-        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,6,3),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,6,3),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,6,3),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="N34" s="17">
-        <f>"4"&amp;CHAR(10)&amp;IFERROR("P: "&amp;VLOOKUP(DATE(2027,6,4),Purple!$A:$J,10,FALSE),IFERROR("G: "&amp;VLOOKUP(DATE(2027,6,4),Gold!$A:$J,10,FALSE),"Exam"))</f>
+        <f>"4"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,6,4),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,6,4),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,6,4),Assessments!$H:$I,2,FALSE),CHAR(10)&amp;"Exam day")</f>
         <v/>
       </c>
       <c r="O34" s="14" t="inlineStr">
@@ -2752,30 +2757,30 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="28" customHeight="1">
+    <row r="35" ht="40" customHeight="1">
       <c r="A35" s="14" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
       <c r="B35" s="16">
-        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,3),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,3),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,3),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C35" s="15">
-        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,4),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,4),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,4),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="D35" s="16">
-        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,5),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,5),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,5),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="E35" s="15">
-        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,6),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,6),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,6),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="F35" s="16">
-        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,7),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,7),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,7),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="G35" s="14" t="inlineStr">
@@ -2789,11 +2794,11 @@
         </is>
       </c>
       <c r="J35" s="17">
-        <f>"7"&amp;CHAR(10)&amp;IFERROR("P: "&amp;VLOOKUP(DATE(2027,6,7),Purple!$A:$J,10,FALSE),IFERROR("G: "&amp;VLOOKUP(DATE(2027,6,7),Gold!$A:$J,10,FALSE),"Exam"))</f>
+        <f>"7"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,6,7),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,6,7),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,6,7),Assessments!$H:$I,2,FALSE),CHAR(10)&amp;"Exam day")</f>
         <v/>
       </c>
       <c r="K35" s="17">
-        <f>"8"&amp;CHAR(10)&amp;IFERROR("P: "&amp;VLOOKUP(DATE(2027,6,8),Purple!$A:$J,10,FALSE),IFERROR("G: "&amp;VLOOKUP(DATE(2027,6,8),Gold!$A:$J,10,FALSE),"Exam"))</f>
+        <f>"8"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,6,8),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,6,8),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,6,8),Assessments!$H:$I,2,FALSE),CHAR(10)&amp;"Exam day")</f>
         <v/>
       </c>
       <c r="L35" s="14" t="inlineStr">
@@ -2817,30 +2822,30 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="28" customHeight="1">
+    <row r="36" ht="40" customHeight="1">
       <c r="A36" s="14" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
       <c r="B36" s="15">
-        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,10),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,10),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,10),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C36" s="16">
-        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,11),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,11),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,11),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="D36" s="15">
-        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,12),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,12),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,12),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="E36" s="16">
-        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,13),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,13),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,13),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="F36" s="15">
-        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,14),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,14),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,14),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="G36" s="14" t="inlineStr">
@@ -2884,30 +2889,30 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="28" customHeight="1">
+    <row r="37" ht="40" customHeight="1">
       <c r="A37" s="14" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
       <c r="B37" s="16">
-        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,17),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,17),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,17),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C37" s="15">
-        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,18),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,18),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,18),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="D37" s="16">
-        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,19),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,19),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,19),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="E37" s="15">
-        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,20),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,20),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,20),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="F37" s="16">
-        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,21),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,21),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,21),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="G37" s="14" t="inlineStr">
@@ -2951,30 +2956,30 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="28" customHeight="1">
+    <row r="38" ht="40" customHeight="1">
       <c r="A38" s="14" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
       <c r="B38" s="15">
-        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,24),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,24),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,24),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C38" s="16">
-        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,25),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,25),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,25),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="D38" s="15">
-        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,26),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,26),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,26),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="E38" s="16">
-        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,27),Gold!$A:$J,10,FALSE),"")</f>
+        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,27),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,27),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="F38" s="18">
-        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,28),Purple!$A:$J,10,FALSE),"")</f>
+        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,28),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,28),Assessments!$H:$I,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="G38" s="14" t="inlineStr">
@@ -3006,7 +3011,7 @@
       <c r="N38" s="13" t="n"/>
       <c r="O38" s="13" t="n"/>
     </row>
-    <row r="39" ht="28" customHeight="1">
+    <row r="39" ht="40" customHeight="1">
       <c r="A39" s="14" t="inlineStr">
         <is>
           <t>30</t>
@@ -7607,7 +7612,7 @@
       </c>
       <c r="E87" s="21" t="inlineStr">
         <is>
-          <t>Q1 Bench</t>
+          <t>Q1 Benchmark</t>
         </is>
       </c>
       <c r="F87" s="21" t="inlineStr">
@@ -7675,7 +7680,7 @@
       </c>
       <c r="E89" s="21" t="inlineStr">
         <is>
-          <t>Q2 Bench</t>
+          <t>Q2 Benchmark</t>
         </is>
       </c>
       <c r="F89" s="21" t="inlineStr">
@@ -7777,7 +7782,7 @@
       </c>
       <c r="E92" s="21" t="inlineStr">
         <is>
-          <t>Q3 Bench</t>
+          <t>Q3 Benchmark</t>
         </is>
       </c>
       <c r="F92" s="21" t="inlineStr">
@@ -7845,7 +7850,7 @@
       </c>
       <c r="E94" s="21" t="inlineStr">
         <is>
-          <t>Q4 Bench</t>
+          <t>Q4 Benchmark</t>
         </is>
       </c>
       <c r="F94" s="21" t="inlineStr">
@@ -16118,7 +16123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16127,6 +16132,9 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="3" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16160,6 +16168,16 @@
           <t>Planned near (unit guide)</t>
         </is>
       </c>
+      <c r="H1" s="19" t="inlineStr">
+        <is>
+          <t>Exam or test date</t>
+        </is>
+      </c>
+      <c r="I1" s="19" t="inlineStr">
+        <is>
+          <t>Exam shown on calendar</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="20" t="inlineStr">
@@ -16184,6 +16202,14 @@
           <t>U1 W4L2: Learn key elements to evaluate clarity and accuracy in infor</t>
         </is>
       </c>
+      <c r="H2" s="31" t="n">
+        <v>46407</v>
+      </c>
+      <c r="I2" s="32" t="inlineStr">
+        <is>
+          <t>Midyear exams: Math, Sci, Soc. St.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="inlineStr">
@@ -16208,6 +16234,14 @@
           <t xml:space="preserve">U2 C3L1: Use my rough draft and my notes to type a final draft of my </t>
         </is>
       </c>
+      <c r="H3" s="31" t="n">
+        <v>46408</v>
+      </c>
+      <c r="I3" s="32" t="inlineStr">
+        <is>
+          <t>Midyear exams: Math, Sci, Soc. St.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
@@ -16232,6 +16266,14 @@
           <t>U3 C2L5: Learn poetic devices, then read and annotate “Siren Song” by</t>
         </is>
       </c>
+      <c r="H4" s="31" t="n">
+        <v>46409</v>
+      </c>
+      <c r="I4" s="32" t="inlineStr">
+        <is>
+          <t>Midyear exams: Math, Sci, Soc. St.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="inlineStr">
@@ -16256,6 +16298,14 @@
           <t>U4 C2L1: Read and analyze The Scarlet Ibis to determine the impact of</t>
         </is>
       </c>
+      <c r="H5" s="31" t="n">
+        <v>46526</v>
+      </c>
+      <c r="I5" s="32" t="inlineStr">
+        <is>
+          <t>Reading SOL</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
@@ -16276,6 +16326,14 @@
         <v>46427</v>
       </c>
       <c r="F6" s="20" t="inlineStr"/>
+      <c r="H6" s="31" t="n">
+        <v>46527</v>
+      </c>
+      <c r="I6" s="32" t="inlineStr">
+        <is>
+          <t>History SOL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="inlineStr">
@@ -16300,6 +16358,14 @@
           <t>U5 C4L1: Explain how characters advance the plot and themes in a nove</t>
         </is>
       </c>
+      <c r="H7" s="31" t="n">
+        <v>46532</v>
+      </c>
+      <c r="I7" s="32" t="inlineStr">
+        <is>
+          <t>Math SOL</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
@@ -16324,6 +16390,14 @@
           <t>U5 C5L2: Examine and analyze the characteristics of literature that c</t>
         </is>
       </c>
+      <c r="H8" s="31" t="n">
+        <v>46533</v>
+      </c>
+      <c r="I8" s="32" t="inlineStr">
+        <is>
+          <t>Science SOL</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="inlineStr">
@@ -16348,6 +16422,14 @@
           <t>U6 C2L4: Plan and organize my writing.</t>
         </is>
       </c>
+      <c r="H9" s="31" t="n">
+        <v>46542</v>
+      </c>
+      <c r="I9" s="32" t="inlineStr">
+        <is>
+          <t>Final exams: Math, Sci, Soc. St.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
@@ -16361,7 +16443,7 @@
       <c r="C10" s="28" t="n">
         <v>46554</v>
       </c>
-      <c r="D10" s="31" t="n">
+      <c r="D10" s="33" t="n">
         <v>46542</v>
       </c>
       <c r="E10" s="30" t="n">
@@ -16372,83 +16454,109 @@
           <t>U7 C2L3: Engage in reading, writing, research, and discussion to exam</t>
         </is>
       </c>
+      <c r="H10" s="31" t="n">
+        <v>46545</v>
+      </c>
+      <c r="I10" s="32" t="inlineStr">
+        <is>
+          <t>Final exams: Math, Sci, Soc. St.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="H11" s="31" t="n">
+        <v>46546</v>
+      </c>
+      <c r="I11" s="32" t="inlineStr">
+        <is>
+          <t>Final exams: Math, Sci, Soc. St.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="32" t="inlineStr">
+      <c r="A12" s="34" t="inlineStr">
         <is>
           <t>Other testing that may pull students (from the NNPS testing calendar)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="33" t="inlineStr">
+      <c r="A13" s="35" t="inlineStr">
         <is>
           <t>LPA (Grade 9 retake)</t>
         </is>
       </c>
-      <c r="B13" s="33" t="inlineStr">
+      <c r="B13" s="35" t="inlineStr">
         <is>
           <t>11/16/2026</t>
         </is>
       </c>
-      <c r="C13" s="33" t="inlineStr">
+      <c r="C13" s="35" t="inlineStr">
         <is>
           <t>11/20/2026</t>
         </is>
       </c>
+      <c r="H13" s="36" t="inlineStr">
+        <is>
+          <t>Edit or add rows here and the Year at a Glance tab updates. The testing calendar does not say which subject is on which exam day; type the subject once the exam schedule is out.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="33" t="inlineStr">
+      <c r="A14" s="35" t="inlineStr">
         <is>
           <t>Fall SOL non-writing</t>
         </is>
       </c>
-      <c r="B14" s="33" t="inlineStr">
+      <c r="B14" s="35" t="inlineStr">
         <is>
           <t>11/30/2026</t>
         </is>
       </c>
-      <c r="C14" s="33" t="inlineStr">
+      <c r="C14" s="35" t="inlineStr">
         <is>
           <t>12/11/2026</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="33" t="inlineStr">
+      <c r="A15" s="35" t="inlineStr">
         <is>
           <t>WIDA</t>
         </is>
       </c>
-      <c r="B15" s="33" t="inlineStr">
+      <c r="B15" s="35" t="inlineStr">
         <is>
           <t>1/11/2027</t>
         </is>
       </c>
-      <c r="C15" s="33" t="inlineStr">
+      <c r="C15" s="35" t="inlineStr">
         <is>
           <t>3/19/2027</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="33" t="inlineStr">
+      <c r="A16" s="35" t="inlineStr">
         <is>
           <t>Expedited retakes, all content</t>
         </is>
       </c>
-      <c r="B16" s="33" t="inlineStr">
+      <c r="B16" s="35" t="inlineStr">
         <is>
           <t>6/1/2027</t>
         </is>
       </c>
-      <c r="C16" s="33" t="inlineStr">
+      <c r="C16" s="35" t="inlineStr">
         <is>
           <t>6/4/2027</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="H13:I15"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Limit the pacing calendar to English exams
Drops the midyear/final exam subjects, SOL dates and non-English testing
windows; only English 9 MQ, benchmark and LPA dates appear.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y9R7PeCARjWUDy39JuMJzQ
</commit_message>
<xml_diff>
--- a/english9-pacing/English9_PurpleGold_Pacing_2026-27.xlsx
+++ b/english9-pacing/English9_PurpleGold_Pacing_2026-27.xlsx
@@ -213,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -299,16 +299,11 @@
     <xf numFmtId="165" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -747,7 +742,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Assessments: where each midquarter, benchmark and LPA landed for each track, inside its testing window. Its yellow Exam table (columns H and I) lists midyear exams, final exams and SOL test dates; each one is printed on its day in Year at a Glance.</t>
+          <t>Assessments: where each midquarter, benchmark and LPA landed for each track, inside its testing window.</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1030,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="40" customHeight="1">
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="13" t="n"/>
       <c r="B7" s="13" t="n"/>
       <c r="C7" s="13" t="n"/>
@@ -1050,15 +1045,15 @@
       <c r="I7" s="13" t="n"/>
       <c r="J7" s="13" t="n"/>
       <c r="K7" s="15">
-        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,1),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,1),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,1),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="L7" s="16">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,2),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,2),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,2),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="M7" s="15">
-        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,3),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,3),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,3),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="N7" s="14" t="inlineStr">
@@ -1076,11 +1071,11 @@
       <c r="S7" s="13" t="n"/>
       <c r="T7" s="13" t="n"/>
       <c r="U7" s="15">
-        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,1),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,1),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,1),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="V7" s="16">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,2),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,2),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,2),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="W7" s="14" t="inlineStr">
@@ -1089,7 +1084,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="40" customHeight="1">
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
           <t>2</t>
@@ -1136,19 +1131,19 @@
         </is>
       </c>
       <c r="K8" s="16">
-        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,8),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,8),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,8),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="L8" s="15">
-        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,9),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,9),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,9),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="M8" s="16">
-        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,10),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,10),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,10),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="N8" s="15">
-        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,11),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,11),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,11),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="O8" s="14" t="inlineStr">
@@ -1162,23 +1157,23 @@
         </is>
       </c>
       <c r="R8" s="15">
-        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,5),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,5),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,5),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="S8" s="16">
-        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,6),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,6),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,6),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="T8" s="15">
-        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,7),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,7),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,7),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="U8" s="16">
-        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,8),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,8),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,8),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="V8" s="15">
-        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,9),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,9),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,9),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="W8" s="14" t="inlineStr">
@@ -1187,7 +1182,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="40" customHeight="1">
+    <row r="9" ht="28" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
           <t>9</t>
@@ -1229,23 +1224,23 @@
         </is>
       </c>
       <c r="J9" s="16">
-        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,14),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,14),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,14),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="K9" s="15">
-        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,15),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,15),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,15),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="L9" s="16">
-        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,16),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,16),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,16),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="M9" s="15">
-        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,17),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,17),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,17),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="N9" s="16">
-        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,18),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,18),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,18),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="O9" s="14" t="inlineStr">
@@ -1259,19 +1254,19 @@
         </is>
       </c>
       <c r="R9" s="16">
-        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,12),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,12),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,12),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="S9" s="15">
-        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,13),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,13),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,13),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="T9" s="16">
-        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,14),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,14),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,14),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="U9" s="15">
-        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,15),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,15),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,15),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="V9" s="14" t="inlineStr">
@@ -1285,7 +1280,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="40" customHeight="1">
+    <row r="10" ht="28" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
           <t>16</t>
@@ -1327,23 +1322,23 @@
         </is>
       </c>
       <c r="J10" s="15">
-        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,21),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,21),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,21),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="K10" s="16">
-        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,22),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,22),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,22),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="L10" s="15">
-        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,23),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,23),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,23),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="M10" s="16">
-        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,24),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,24),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,24),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="N10" s="15">
-        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,25),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,25),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,25),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="O10" s="14" t="inlineStr">
@@ -1357,23 +1352,23 @@
         </is>
       </c>
       <c r="R10" s="16">
-        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,19),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,19),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,19),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="S10" s="15">
-        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,20),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,20),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,20),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="T10" s="16">
-        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,21),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,21),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,21),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="U10" s="15">
-        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,22),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,22),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,22),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="V10" s="16">
-        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,23),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,23),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,23),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="W10" s="14" t="inlineStr">
@@ -1382,30 +1377,30 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="40" customHeight="1">
+    <row r="11" ht="28" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
       <c r="B11" s="15">
-        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,24),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,8,24),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,24),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="C11" s="16">
-        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,25),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,8,25),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,25),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="D11" s="15">
-        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,26),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,8,26),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,26),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="E11" s="16">
-        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,27),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,8,27),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,27),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="F11" s="15">
-        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,28),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,8,28),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,28),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="G11" s="14" t="inlineStr">
@@ -1419,15 +1414,15 @@
         </is>
       </c>
       <c r="J11" s="16">
-        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,28),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,28),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,28),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="K11" s="15">
-        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,29),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,29),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,29),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="L11" s="16">
-        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,30),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,9,30),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,9,30),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="M11" s="13" t="n"/>
@@ -1439,23 +1434,23 @@
         </is>
       </c>
       <c r="R11" s="15">
-        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,26),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,26),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,26),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="S11" s="16">
-        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,27),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,27),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,27),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="T11" s="15">
-        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,28),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,28),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,28),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="U11" s="16">
-        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,29),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,29),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,29),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="V11" s="15">
-        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,30),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,10,30),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,10,30),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="W11" s="14" t="inlineStr">
@@ -1464,14 +1459,14 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="40" customHeight="1">
+    <row r="12" ht="28" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
       <c r="B12" s="16">
-        <f>"31"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,31),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,8,31),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"31"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,8,31),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="C12" s="13" t="n"/>
@@ -1618,14 +1613,14 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="40" customHeight="1">
+    <row r="16" ht="28" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="B16" s="16">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,2),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,2),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,2),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="C16" s="14" t="inlineStr">
@@ -1634,15 +1629,15 @@
         </is>
       </c>
       <c r="D16" s="15">
-        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,4),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,4),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,4),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="E16" s="16">
-        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,5),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,5),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,5),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,6),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,6),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,6),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="G16" s="14" t="inlineStr">
@@ -1653,19 +1648,19 @@
       <c r="I16" s="13" t="n"/>
       <c r="J16" s="13" t="n"/>
       <c r="K16" s="15">
-        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,1),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,1),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,1),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="L16" s="16">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,2),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,2),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,2),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="M16" s="15">
-        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,3),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,3),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,3),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="N16" s="16">
-        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,4),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,4),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,4),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="O16" s="14" t="inlineStr">
@@ -1689,30 +1684,30 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="40" customHeight="1">
+    <row r="17" ht="28" customHeight="1">
       <c r="A17" s="14" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
       <c r="B17" s="16">
-        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,9),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,9),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,9),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="C17" s="15">
-        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,10),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,10),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,10),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="D17" s="16">
-        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,11),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,11),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,11),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="E17" s="15">
-        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,12),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,12),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,12),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="F17" s="16">
-        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,13),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,13),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,13),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="G17" s="14" t="inlineStr">
@@ -1726,23 +1721,23 @@
         </is>
       </c>
       <c r="J17" s="15">
-        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,7),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,7),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,7),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="K17" s="16">
-        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,8),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,8),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,8),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="L17" s="15">
-        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,9),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,9),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,9),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="M17" s="16">
-        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,10),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,10),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,10),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="N17" s="15">
-        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,11),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,11),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,11),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="O17" s="14" t="inlineStr">
@@ -1761,19 +1756,19 @@
         </is>
       </c>
       <c r="S17" s="15">
-        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,5),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,5),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,5),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="T17" s="16">
-        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,6),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,6),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,6),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="U17" s="15">
-        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,7),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,7),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,7),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="V17" s="16">
-        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,8),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,8),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,8),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="W17" s="14" t="inlineStr">
@@ -1782,30 +1777,30 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="40" customHeight="1">
+    <row r="18" ht="28" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
       <c r="B18" s="15">
-        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,16),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,16),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,16),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="C18" s="16">
-        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,17),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,17),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,17),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="D18" s="15">
-        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,18),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,18),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,18),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="E18" s="16">
-        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,19),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,19),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,19),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="F18" s="15">
-        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,20),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,20),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,20),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="G18" s="14" t="inlineStr">
@@ -1819,23 +1814,23 @@
         </is>
       </c>
       <c r="J18" s="16">
-        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,14),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,14),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,14),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="K18" s="15">
-        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,15),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,15),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,15),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="L18" s="16">
-        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,16),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,16),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,16),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="M18" s="15">
-        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,17),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,17),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,17),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="N18" s="16">
-        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,18),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,12,18),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,12,18),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="O18" s="14" t="inlineStr">
@@ -1849,23 +1844,23 @@
         </is>
       </c>
       <c r="R18" s="15">
-        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,11),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,11),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,11),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="S18" s="16">
-        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,12),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,12),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,12),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="T18" s="15">
-        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,13),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,13),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,13),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="U18" s="16">
-        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,14),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,14),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,14),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="V18" s="15">
-        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,15),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,15),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,15),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="W18" s="14" t="inlineStr">
@@ -1874,18 +1869,18 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="40" customHeight="1">
+    <row r="19" ht="28" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
       <c r="B19" s="16">
-        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,23),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,23),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,23),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="C19" s="15">
-        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,24),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,24),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,24),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="D19" s="14" t="inlineStr">
@@ -1954,19 +1949,19 @@
         </is>
       </c>
       <c r="S19" s="16">
-        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,19),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,19),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,19),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="T19" s="17">
-        <f>"20"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,1,20),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,1,20),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,20),Assessments!$H:$I,2,FALSE),CHAR(10)&amp;"Exam day")</f>
+        <f>"20"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,1,20),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,1,20),Gold!$A:$J,10,FALSE),"")&amp;IF(COUNTIF(Purple!$A:$A,DATE(2027,1,20))+COUNTIF(Gold!$A:$A,DATE(2027,1,20))=0,CHAR(10)&amp;"Exam day","")</f>
         <v/>
       </c>
       <c r="U19" s="17">
-        <f>"21"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,1,21),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,1,21),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,21),Assessments!$H:$I,2,FALSE),CHAR(10)&amp;"Exam day")</f>
+        <f>"21"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,1,21),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,1,21),Gold!$A:$J,10,FALSE),"")&amp;IF(COUNTIF(Purple!$A:$A,DATE(2027,1,21))+COUNTIF(Gold!$A:$A,DATE(2027,1,21))=0,CHAR(10)&amp;"Exam day","")</f>
         <v/>
       </c>
       <c r="V19" s="17">
-        <f>"22"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,1,22),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,1,22),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,22),Assessments!$H:$I,2,FALSE),CHAR(10)&amp;"Exam day")</f>
+        <f>"22"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,1,22),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,1,22),Gold!$A:$J,10,FALSE),"")&amp;IF(COUNTIF(Purple!$A:$A,DATE(2027,1,22))+COUNTIF(Gold!$A:$A,DATE(2027,1,22))=0,CHAR(10)&amp;"Exam day","")</f>
         <v/>
       </c>
       <c r="W19" s="14" t="inlineStr">
@@ -1975,14 +1970,14 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="40" customHeight="1">
+    <row r="20" ht="28" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
       <c r="B20" s="16">
-        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,30),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2026,11,30),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2026,11,30),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="C20" s="13" t="n"/>
@@ -2033,15 +2028,15 @@
         </is>
       </c>
       <c r="T20" s="15">
-        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,27),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,27),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,27),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="U20" s="16">
-        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,28),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,28),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,28),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="V20" s="15">
-        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,29),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,1,29),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,1,29),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="W20" s="14" t="inlineStr">
@@ -2050,7 +2045,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="40" customHeight="1">
+    <row r="21" ht="28" customHeight="1">
       <c r="A21" s="13" t="n"/>
       <c r="B21" s="13" t="n"/>
       <c r="C21" s="13" t="n"/>
@@ -2201,26 +2196,26 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="40" customHeight="1">
+    <row r="25" ht="28" customHeight="1">
       <c r="A25" s="13" t="n"/>
       <c r="B25" s="16">
-        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,1),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,1),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,1),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="C25" s="15">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,2),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,2),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,2),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="D25" s="16">
-        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,3),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,3),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,3),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="E25" s="15">
-        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,4),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,4),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,4),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="F25" s="16">
-        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,5),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,5),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,5),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="G25" s="14" t="inlineStr">
@@ -2230,23 +2225,23 @@
       </c>
       <c r="I25" s="13" t="n"/>
       <c r="J25" s="15">
-        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,1),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,1),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,1),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="K25" s="16">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,2),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,2),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,2),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="L25" s="15">
-        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,3),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,3),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,3),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="M25" s="16">
-        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,4),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,4),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,4),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="N25" s="18">
-        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,5),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,5),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,5),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="O25" s="14" t="inlineStr">
@@ -2259,11 +2254,11 @@
       <c r="S25" s="13" t="n"/>
       <c r="T25" s="13" t="n"/>
       <c r="U25" s="16">
-        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,1),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,1),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,1),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="V25" s="18">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,2),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,2),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,2),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="W25" s="14" t="inlineStr">
@@ -2272,30 +2267,30 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="40" customHeight="1">
+    <row r="26" ht="28" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
       <c r="B26" s="15">
-        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,8),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,8),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,8),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="C26" s="16">
-        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,9),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,9),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,9),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="D26" s="15">
-        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,10),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,10),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,10),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="E26" s="16">
-        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,11),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,11),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,11),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="F26" s="15">
-        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,12),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,12),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,12),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="G26" s="14" t="inlineStr">
@@ -2309,23 +2304,23 @@
         </is>
       </c>
       <c r="J26" s="16">
-        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,8),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,8),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"8"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,8),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="K26" s="15">
-        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,9),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,9),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"9"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,9),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="L26" s="16">
-        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,10),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,10),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,10),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="M26" s="15">
-        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,11),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,11),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,11),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="N26" s="16">
-        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,12),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,12),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,12),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="O26" s="14" t="inlineStr">
@@ -2369,7 +2364,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="40" customHeight="1">
+    <row r="27" ht="28" customHeight="1">
       <c r="A27" s="14" t="inlineStr">
         <is>
           <t>14</t>
@@ -2381,19 +2376,19 @@
         </is>
       </c>
       <c r="C27" s="16">
-        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,16),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,16),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,16),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="D27" s="15">
-        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,17),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,17),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,17),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="E27" s="16">
-        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,18),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,18),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,18),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="F27" s="15">
-        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,19),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,19),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,19),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="G27" s="14" t="inlineStr">
@@ -2407,23 +2402,23 @@
         </is>
       </c>
       <c r="J27" s="15">
-        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,15),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,15),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,15),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="K27" s="16">
-        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,16),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,16),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,16),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="L27" s="15">
-        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,17),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,17),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,17),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="M27" s="16">
-        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,18),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,18),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,18),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="N27" s="15">
-        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,19),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,19),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,19),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="O27" s="14" t="inlineStr">
@@ -2442,19 +2437,19 @@
         </is>
       </c>
       <c r="S27" s="16">
-        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,13),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,13),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,13),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="T27" s="15">
-        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,14),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,14),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,14),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="U27" s="16">
-        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,15),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,15),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"15"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,15),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="V27" s="15">
-        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,16),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,16),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"16"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,16),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="W27" s="14" t="inlineStr">
@@ -2463,30 +2458,30 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="40" customHeight="1">
+    <row r="28" ht="28" customHeight="1">
       <c r="A28" s="14" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
       <c r="B28" s="16">
-        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,22),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,22),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,22),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="C28" s="15">
-        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,23),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,23),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,23),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="D28" s="16">
-        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,24),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,24),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,24),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="E28" s="15">
-        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,25),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,25),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,25),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="F28" s="16">
-        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,26),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,2,26),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,2,26),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="G28" s="14" t="inlineStr">
@@ -2500,23 +2495,23 @@
         </is>
       </c>
       <c r="J28" s="16">
-        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,22),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,22),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,22),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="K28" s="15">
-        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,23),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,23),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,23),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="L28" s="16">
-        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,24),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,24),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,24),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="M28" s="15">
-        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,25),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,25),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,25),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="N28" s="16">
-        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,26),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,26),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,26),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="O28" s="14" t="inlineStr">
@@ -2530,23 +2525,23 @@
         </is>
       </c>
       <c r="R28" s="16">
-        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,19),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,19),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,19),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="S28" s="15">
-        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,20),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,20),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,20),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="T28" s="16">
-        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,21),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,21),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,21),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="U28" s="15">
-        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,22),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,22),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"22"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,22),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="V28" s="16">
-        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,23),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,23),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"23"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,23),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="W28" s="14" t="inlineStr">
@@ -2555,7 +2550,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="40" customHeight="1">
+    <row r="29" ht="28" customHeight="1">
       <c r="A29" s="14" t="inlineStr">
         <is>
           <t>28</t>
@@ -2573,15 +2568,15 @@
         </is>
       </c>
       <c r="J29" s="15">
-        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,29),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,29),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,29),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="K29" s="16">
-        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,30),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,30),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,30),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="L29" s="15">
-        <f>"31"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,31),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,3,31),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"31"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,3,31),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="M29" s="13" t="n"/>
@@ -2593,28 +2588,28 @@
         </is>
       </c>
       <c r="R29" s="15">
-        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,26),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,26),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,26),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="S29" s="16">
-        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,27),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,27),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,27),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="T29" s="15">
-        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,28),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,28),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,28),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="U29" s="16">
-        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,29),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,29),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"29"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,29),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="V29" s="15">
-        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,30),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,4,30),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"30"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,4,30),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="W29" s="13" t="n"/>
     </row>
-    <row r="30" ht="40" customHeight="1">
+    <row r="30" ht="28" customHeight="1">
       <c r="A30" s="13" t="n"/>
       <c r="B30" s="13" t="n"/>
       <c r="C30" s="13" t="n"/>
@@ -2721,7 +2716,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="40" customHeight="1">
+    <row r="34" ht="28" customHeight="1">
       <c r="A34" s="13" t="n"/>
       <c r="B34" s="13" t="n"/>
       <c r="C34" s="13" t="n"/>
@@ -2736,19 +2731,19 @@
       <c r="I34" s="13" t="n"/>
       <c r="J34" s="13" t="n"/>
       <c r="K34" s="16">
-        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,6,1),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,6,1),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"1"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,6,1),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="L34" s="15">
-        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,6,2),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,6,2),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"2"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,6,2),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="M34" s="16">
-        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,6,3),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,6,3),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,6,3),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="N34" s="17">
-        <f>"4"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,6,4),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,6,4),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,6,4),Assessments!$H:$I,2,FALSE),CHAR(10)&amp;"Exam day")</f>
+        <f>"4"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,6,4),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,6,4),Gold!$A:$J,10,FALSE),"")&amp;IF(COUNTIF(Purple!$A:$A,DATE(2027,6,4))+COUNTIF(Gold!$A:$A,DATE(2027,6,4))=0,CHAR(10)&amp;"Exam day","")</f>
         <v/>
       </c>
       <c r="O34" s="14" t="inlineStr">
@@ -2757,30 +2752,30 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="40" customHeight="1">
+    <row r="35" ht="28" customHeight="1">
       <c r="A35" s="14" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
       <c r="B35" s="16">
-        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,3),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,3),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"3"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,3),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="C35" s="15">
-        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,4),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,4),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"4"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,4),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="D35" s="16">
-        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,5),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,5),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"5"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,5),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="E35" s="15">
-        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,6),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,6),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"6"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,6),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="F35" s="16">
-        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,7),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,7),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"7"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,7),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="G35" s="14" t="inlineStr">
@@ -2794,11 +2789,11 @@
         </is>
       </c>
       <c r="J35" s="17">
-        <f>"7"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,6,7),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,6,7),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,6,7),Assessments!$H:$I,2,FALSE),CHAR(10)&amp;"Exam day")</f>
+        <f>"7"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,6,7),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,6,7),Gold!$A:$J,10,FALSE),"")&amp;IF(COUNTIF(Purple!$A:$A,DATE(2027,6,7))+COUNTIF(Gold!$A:$A,DATE(2027,6,7))=0,CHAR(10)&amp;"Exam day","")</f>
         <v/>
       </c>
       <c r="K35" s="17">
-        <f>"8"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,6,8),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,6,8),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,6,8),Assessments!$H:$I,2,FALSE),CHAR(10)&amp;"Exam day")</f>
+        <f>"8"&amp;IFERROR(CHAR(10)&amp;"P: "&amp;VLOOKUP(DATE(2027,6,8),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;"G: "&amp;VLOOKUP(DATE(2027,6,8),Gold!$A:$J,10,FALSE),"")&amp;IF(COUNTIF(Purple!$A:$A,DATE(2027,6,8))+COUNTIF(Gold!$A:$A,DATE(2027,6,8))=0,CHAR(10)&amp;"Exam day","")</f>
         <v/>
       </c>
       <c r="L35" s="14" t="inlineStr">
@@ -2822,30 +2817,30 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="40" customHeight="1">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="14" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
       <c r="B36" s="15">
-        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,10),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,10),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"10"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,10),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="C36" s="16">
-        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,11),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,11),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"11"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,11),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="D36" s="15">
-        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,12),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,12),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"12"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,12),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="E36" s="16">
-        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,13),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,13),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"13"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,13),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="F36" s="15">
-        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,14),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,14),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"14"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,14),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="G36" s="14" t="inlineStr">
@@ -2889,30 +2884,30 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="40" customHeight="1">
+    <row r="37" ht="28" customHeight="1">
       <c r="A37" s="14" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
       <c r="B37" s="16">
-        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,17),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,17),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"17"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,17),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="C37" s="15">
-        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,18),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,18),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"18"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,18),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="D37" s="16">
-        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,19),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,19),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"19"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,19),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="E37" s="15">
-        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,20),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,20),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"20"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,20),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="F37" s="16">
-        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,21),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,21),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"21"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,21),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="G37" s="14" t="inlineStr">
@@ -2956,30 +2951,30 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="40" customHeight="1">
+    <row r="38" ht="28" customHeight="1">
       <c r="A38" s="14" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
       <c r="B38" s="15">
-        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,24),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,24),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"24"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,24),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="C38" s="16">
-        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,25),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,25),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"25"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,25),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="D38" s="15">
-        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,26),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,26),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"26"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,26),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="E38" s="16">
-        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,27),Gold!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,27),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"27"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,27),Gold!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="F38" s="18">
-        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,28),Purple!$A:$J,10,FALSE),"")&amp;IFERROR(CHAR(10)&amp;VLOOKUP(DATE(2027,5,28),Assessments!$H:$I,2,FALSE),"")</f>
+        <f>"28"&amp;CHAR(10)&amp;IFERROR(VLOOKUP(DATE(2027,5,28),Purple!$A:$J,10,FALSE),"")</f>
         <v/>
       </c>
       <c r="G38" s="14" t="inlineStr">
@@ -3011,7 +3006,7 @@
       <c r="N38" s="13" t="n"/>
       <c r="O38" s="13" t="n"/>
     </row>
-    <row r="39" ht="40" customHeight="1">
+    <row r="39" ht="28" customHeight="1">
       <c r="A39" s="14" t="inlineStr">
         <is>
           <t>30</t>
@@ -16123,7 +16118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -16132,9 +16127,6 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="3" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16168,16 +16160,6 @@
           <t>Planned near (unit guide)</t>
         </is>
       </c>
-      <c r="H1" s="19" t="inlineStr">
-        <is>
-          <t>Exam or test date</t>
-        </is>
-      </c>
-      <c r="I1" s="19" t="inlineStr">
-        <is>
-          <t>Exam shown on calendar</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="20" t="inlineStr">
@@ -16202,14 +16184,6 @@
           <t>U1 W4L2: Learn key elements to evaluate clarity and accuracy in infor</t>
         </is>
       </c>
-      <c r="H2" s="31" t="n">
-        <v>46407</v>
-      </c>
-      <c r="I2" s="32" t="inlineStr">
-        <is>
-          <t>Midyear exams: Math, Sci, Soc. St.</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="inlineStr">
@@ -16234,14 +16208,6 @@
           <t xml:space="preserve">U2 C3L1: Use my rough draft and my notes to type a final draft of my </t>
         </is>
       </c>
-      <c r="H3" s="31" t="n">
-        <v>46408</v>
-      </c>
-      <c r="I3" s="32" t="inlineStr">
-        <is>
-          <t>Midyear exams: Math, Sci, Soc. St.</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
@@ -16266,14 +16232,6 @@
           <t>U3 C2L5: Learn poetic devices, then read and annotate “Siren Song” by</t>
         </is>
       </c>
-      <c r="H4" s="31" t="n">
-        <v>46409</v>
-      </c>
-      <c r="I4" s="32" t="inlineStr">
-        <is>
-          <t>Midyear exams: Math, Sci, Soc. St.</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="inlineStr">
@@ -16298,14 +16256,6 @@
           <t>U4 C2L1: Read and analyze The Scarlet Ibis to determine the impact of</t>
         </is>
       </c>
-      <c r="H5" s="31" t="n">
-        <v>46526</v>
-      </c>
-      <c r="I5" s="32" t="inlineStr">
-        <is>
-          <t>Reading SOL</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
@@ -16326,14 +16276,6 @@
         <v>46427</v>
       </c>
       <c r="F6" s="20" t="inlineStr"/>
-      <c r="H6" s="31" t="n">
-        <v>46527</v>
-      </c>
-      <c r="I6" s="32" t="inlineStr">
-        <is>
-          <t>History SOL</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="inlineStr">
@@ -16358,14 +16300,6 @@
           <t>U5 C4L1: Explain how characters advance the plot and themes in a nove</t>
         </is>
       </c>
-      <c r="H7" s="31" t="n">
-        <v>46532</v>
-      </c>
-      <c r="I7" s="32" t="inlineStr">
-        <is>
-          <t>Math SOL</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
@@ -16390,14 +16324,6 @@
           <t>U5 C5L2: Examine and analyze the characteristics of literature that c</t>
         </is>
       </c>
-      <c r="H8" s="31" t="n">
-        <v>46533</v>
-      </c>
-      <c r="I8" s="32" t="inlineStr">
-        <is>
-          <t>Science SOL</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="inlineStr">
@@ -16422,14 +16348,6 @@
           <t>U6 C2L4: Plan and organize my writing.</t>
         </is>
       </c>
-      <c r="H9" s="31" t="n">
-        <v>46542</v>
-      </c>
-      <c r="I9" s="32" t="inlineStr">
-        <is>
-          <t>Final exams: Math, Sci, Soc. St.</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
@@ -16443,7 +16361,7 @@
       <c r="C10" s="28" t="n">
         <v>46554</v>
       </c>
-      <c r="D10" s="33" t="n">
+      <c r="D10" s="31" t="n">
         <v>46542</v>
       </c>
       <c r="E10" s="30" t="n">
@@ -16454,109 +16372,32 @@
           <t>U7 C2L3: Engage in reading, writing, research, and discussion to exam</t>
         </is>
       </c>
-      <c r="H10" s="31" t="n">
-        <v>46545</v>
-      </c>
-      <c r="I10" s="32" t="inlineStr">
-        <is>
-          <t>Final exams: Math, Sci, Soc. St.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="H11" s="31" t="n">
-        <v>46546</v>
-      </c>
-      <c r="I11" s="32" t="inlineStr">
-        <is>
-          <t>Final exams: Math, Sci, Soc. St.</t>
-        </is>
-      </c>
     </row>
     <row r="12">
-      <c r="A12" s="34" t="inlineStr">
-        <is>
-          <t>Other testing that may pull students (from the NNPS testing calendar)</t>
+      <c r="A12" s="32" t="inlineStr">
+        <is>
+          <t>Other English testing (from the NNPS testing calendar)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="35" t="inlineStr">
-        <is>
-          <t>LPA (Grade 9 retake)</t>
-        </is>
-      </c>
-      <c r="B13" s="35" t="inlineStr">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>LPA (Grade 9 retake, students who need it)</t>
+        </is>
+      </c>
+      <c r="B13" s="33" t="inlineStr">
         <is>
           <t>11/16/2026</t>
         </is>
       </c>
-      <c r="C13" s="35" t="inlineStr">
+      <c r="C13" s="33" t="inlineStr">
         <is>
           <t>11/20/2026</t>
         </is>
       </c>
-      <c r="H13" s="36" t="inlineStr">
-        <is>
-          <t>Edit or add rows here and the Year at a Glance tab updates. The testing calendar does not say which subject is on which exam day; type the subject once the exam schedule is out.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="35" t="inlineStr">
-        <is>
-          <t>Fall SOL non-writing</t>
-        </is>
-      </c>
-      <c r="B14" s="35" t="inlineStr">
-        <is>
-          <t>11/30/2026</t>
-        </is>
-      </c>
-      <c r="C14" s="35" t="inlineStr">
-        <is>
-          <t>12/11/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="35" t="inlineStr">
-        <is>
-          <t>WIDA</t>
-        </is>
-      </c>
-      <c r="B15" s="35" t="inlineStr">
-        <is>
-          <t>1/11/2027</t>
-        </is>
-      </c>
-      <c r="C15" s="35" t="inlineStr">
-        <is>
-          <t>3/19/2027</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="35" t="inlineStr">
-        <is>
-          <t>Expedited retakes, all content</t>
-        </is>
-      </c>
-      <c r="B16" s="35" t="inlineStr">
-        <is>
-          <t>6/1/2027</t>
-        </is>
-      </c>
-      <c r="C16" s="35" t="inlineStr">
-        <is>
-          <t>6/4/2027</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="H13:I15"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>